<commit_message>
added Nisol Intelligence module
</commit_message>
<xml_diff>
--- a/Documents/Phase_1_AI_Audit_Cost_Calculator.xlsx
+++ b/Documents/Phase_1_AI_Audit_Cost_Calculator.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ssooraj\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Nisol-Labs\Code\Anti-Gravity-Code\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5C66B39-428D-407B-857D-FCD689E49D72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B047DE13-DD63-46AF-8BFA-D23C23AAA5FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cost Calculator" sheetId="1" r:id="rId1"/>
@@ -212,7 +212,7 @@
   <numFmts count="3">
     <numFmt numFmtId="6" formatCode="&quot;₹&quot;\ #,##0;[Red]&quot;₹&quot;\ \-#,##0"/>
     <numFmt numFmtId="164" formatCode="\₹#,##0"/>
-    <numFmt numFmtId="166" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    <numFmt numFmtId="165" formatCode="&quot;₹&quot;\ #,##0.00"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -364,13 +364,13 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="6" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="6" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -718,7 +718,7 @@
       <c r="B5" s="4">
         <v>45000</v>
       </c>
-      <c r="C5" s="20">
+      <c r="C5" s="17">
         <f>B5</f>
         <v>45000</v>
       </c>
@@ -731,7 +731,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="7">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>8</v>
@@ -791,8 +791,7 @@
         <v>50</v>
       </c>
       <c r="C10" s="5">
-        <f>VLOOKUP(B10, 'Lookup Tables'!D2:E4, 2, FALSE)</f>
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>21</v>
@@ -806,20 +805,19 @@
         <v>23</v>
       </c>
       <c r="C11" s="5">
-        <f>VLOOKUP(B11, 'Lookup Tables'!G2:H3, 2, FALSE)</f>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
@@ -827,7 +825,7 @@
       </c>
       <c r="B14" s="9">
         <f>ROUNDUP((B6 + (B8 * 1.2) + (B9 * 0.5)) * C7, 0)</f>
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>27</v>
@@ -842,7 +840,7 @@
       </c>
       <c r="B15" s="10">
         <f>B14 * B5</f>
-        <v>630000</v>
+        <v>540000</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>30</v>
@@ -857,7 +855,7 @@
       </c>
       <c r="B16" s="10">
         <f>B15 * (C10 - 1)</f>
-        <v>0</v>
+        <v>162000.00000000003</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>30</v>
@@ -872,7 +870,7 @@
       </c>
       <c r="B17" s="10">
         <f>B15 * (C11 - 1)</f>
-        <v>0</v>
+        <v>270000</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>30</v>
@@ -887,7 +885,7 @@
       </c>
       <c r="B18" s="12">
         <f>ROUNDUP((B15 * C10 * C11), -3)</f>
-        <v>630000</v>
+        <v>1053000</v>
       </c>
       <c r="C18" s="13" t="s">
         <v>30</v>
@@ -897,12 +895,12 @@
       </c>
     </row>
     <row r="20" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="17" t="s">
+      <c r="A20" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
@@ -910,7 +908,7 @@
       </c>
       <c r="B21" s="15">
         <f>B18 * 0.3</f>
-        <v>189000</v>
+        <v>315900</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>30</v>
@@ -925,7 +923,7 @@
       </c>
       <c r="B22" s="15">
         <f>B18 * 0.4</f>
-        <v>252000</v>
+        <v>421200</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>30</v>
@@ -940,7 +938,7 @@
       </c>
       <c r="B23" s="15">
         <f>B18 * 0.3</f>
-        <v>189000</v>
+        <v>315900</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>30</v>
@@ -1091,7 +1089,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" s="21">
+      <c r="A8" s="18">
         <v>25000</v>
       </c>
       <c r="C8">
@@ -1099,7 +1097,7 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" s="21">
+      <c r="A9" s="18">
         <v>30000</v>
       </c>
       <c r="C9">
@@ -1107,7 +1105,7 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="21">
+      <c r="A10" s="18">
         <v>35000</v>
       </c>
       <c r="C10">
@@ -1115,7 +1113,7 @@
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" s="21">
+      <c r="A11" s="18">
         <v>40000</v>
       </c>
       <c r="C11">
@@ -1123,7 +1121,7 @@
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A12" s="21">
+      <c r="A12" s="18">
         <v>45000</v>
       </c>
       <c r="C12">
@@ -1131,7 +1129,7 @@
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A13" s="21">
+      <c r="A13" s="18">
         <v>50000</v>
       </c>
       <c r="C13">
@@ -1139,7 +1137,7 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A14" s="21">
+      <c r="A14" s="18">
         <v>55000</v>
       </c>
       <c r="C14">
@@ -1147,7 +1145,7 @@
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A15" s="21">
+      <c r="A15" s="18">
         <v>60000</v>
       </c>
       <c r="C15">
@@ -1155,7 +1153,7 @@
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A16" s="21">
+      <c r="A16" s="18">
         <v>65000</v>
       </c>
       <c r="C16">
@@ -1163,7 +1161,7 @@
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" s="21">
+      <c r="A17" s="18">
         <v>70000</v>
       </c>
       <c r="C17">
@@ -1171,8 +1169,11 @@
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A18" s="21">
+      <c r="A18" s="18">
         <v>75000</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>